<commit_message>
Deploy: Updated dashboard logic fixes, added quantity column (then removed per request), and organized data for Streamlit Cloud
</commit_message>
<xml_diff>
--- a/MOMENTUM_DB_2 copy/Stocks/Nifty_500_2025_Apr_20_stocks_results/master_momentum_summary.xlsx
+++ b/MOMENTUM_DB_2 copy/Stocks/Nifty_500_2025_Apr_20_stocks_results/master_momentum_summary.xlsx
@@ -3586,12 +3586,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>INE302A01020</t>
+          <t>INE003A01024</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>EXIDEIND</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -3606,12 +3606,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>INE003A01024</t>
+          <t>INE302A01020</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>EXIDEIND</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -3806,12 +3806,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>INE324A01032</t>
+          <t>INE242C01024</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>JINDALSAW</t>
+          <t>ANANTRAJ</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -3826,12 +3826,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>INE242C01024</t>
+          <t>INE324A01032</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>ANANTRAJ</t>
+          <t>JINDALSAW</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -4286,12 +4286,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>INE463V01026</t>
+          <t>INE732I01013</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>ANANDRATHI</t>
+          <t>ANGELONE</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -4306,12 +4306,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>INE732I01013</t>
+          <t>INE463V01026</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ANGELONE</t>
+          <t>ANANDRATHI</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -4706,12 +4706,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>INE292B01021</t>
+          <t>INE134E01011</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>HBLENGINE</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -4726,12 +4726,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>INE134E01011</t>
+          <t>INE292B01021</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>HBLENGINE</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -5486,12 +5486,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>INE257A01026</t>
+          <t>INE103A01014</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>BHEL</t>
+          <t>MRPL</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -5506,12 +5506,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>INE103A01014</t>
+          <t>INE257A01026</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>MRPL</t>
+          <t>BHEL</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -5846,12 +5846,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>INE903U01023</t>
+          <t>INE040H01021</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>SIGNATURE</t>
+          <t>SUZLON</t>
         </is>
       </c>
       <c r="D272" t="n">
@@ -5866,12 +5866,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>INE040H01021</t>
+          <t>INE903U01023</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>SUZLON</t>
+          <t>SIGNATURE</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -6746,12 +6746,12 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>INE298A01020</t>
+          <t>INE274J01014</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>OIL</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -6786,12 +6786,12 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>INE274J01014</t>
+          <t>INE298A01020</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>OIL</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="D319" t="n">
@@ -7006,12 +7006,12 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>INE094A01015</t>
+          <t>INE271C01023</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>DLF</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -7026,12 +7026,12 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>INE271C01023</t>
+          <t>INE094A01015</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>DLF</t>
+          <t>HINDPETRO</t>
         </is>
       </c>
       <c r="D331" t="n">
@@ -7526,12 +7526,12 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>INE226A01021</t>
+          <t>INE066P01011</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>VOLTAS</t>
+          <t>INOXWIND</t>
         </is>
       </c>
       <c r="D356" t="n">
@@ -7546,12 +7546,12 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>INE066P01011</t>
+          <t>INE114A01011</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>INOXWIND</t>
+          <t>SAIL</t>
         </is>
       </c>
       <c r="D357" t="n">
@@ -7566,12 +7566,12 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>INE114A01011</t>
+          <t>INE226A01021</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>SAIL</t>
+          <t>VOLTAS</t>
         </is>
       </c>
       <c r="D358" t="n">
@@ -7846,12 +7846,12 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>INE226A01021</t>
+          <t>INE274J01014</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>VOLTAS</t>
+          <t>OIL</t>
         </is>
       </c>
       <c r="D372" t="n">
@@ -7866,12 +7866,12 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>INE257A01026</t>
+          <t>INE226A01021</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>BHEL</t>
+          <t>VOLTAS</t>
         </is>
       </c>
       <c r="D373" t="n">
@@ -7886,12 +7886,12 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>INE274J01014</t>
+          <t>INE257A01026</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>OIL</t>
+          <t>BHEL</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -9166,12 +9166,12 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>INE121J01017</t>
+          <t>INE205A01025</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>INDUSTOWER</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="D438" t="n">
@@ -9186,12 +9186,12 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>INE205A01025</t>
+          <t>INE121J01017</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>INDUSTOWER</t>
         </is>
       </c>
       <c r="D439" t="n">
@@ -9506,12 +9506,12 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>INE226A01021</t>
+          <t>INE373A01013</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>VOLTAS</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="D455" t="n">
@@ -9526,12 +9526,12 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>INE373A01013</t>
+          <t>INE226A01021</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>VOLTAS</t>
         </is>
       </c>
       <c r="D456" t="n">
@@ -10006,12 +10006,12 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>INE602A01031</t>
+          <t>INE205C01021</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>PCBL</t>
+          <t>POLYMED</t>
         </is>
       </c>
       <c r="D480" t="n">
@@ -10026,12 +10026,12 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>INE205C01021</t>
+          <t>INE602A01031</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>POLYMED</t>
+          <t>PCBL</t>
         </is>
       </c>
       <c r="D481" t="n">
@@ -12806,12 +12806,12 @@
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>INE090A01021</t>
+          <t>INE704P01025</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>COCHINSHIP</t>
         </is>
       </c>
       <c r="D620" t="n">
@@ -12826,12 +12826,12 @@
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>INE704P01025</t>
+          <t>INE513A01022</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>COCHINSHIP</t>
+          <t>SCHAEFFLER</t>
         </is>
       </c>
       <c r="D621" t="n">
@@ -13326,12 +13326,12 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>INE463V01026</t>
+          <t>INE206F01022</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>ANANDRATHI</t>
+          <t>AIIL</t>
         </is>
       </c>
       <c r="D646" t="n">
@@ -13346,12 +13346,12 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>INE206F01022</t>
+          <t>INE463V01026</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>AIIL</t>
+          <t>ANANDRATHI</t>
         </is>
       </c>
       <c r="D647" t="n">
@@ -13546,12 +13546,12 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>INE935A01035</t>
+          <t>INE982J01020</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>GLENMARK</t>
+          <t>PAYTM</t>
         </is>
       </c>
       <c r="D657" t="n">
@@ -13566,12 +13566,12 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>INE982J01020</t>
+          <t>INE935A01035</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
         <is>
-          <t>PAYTM</t>
+          <t>GLENMARK</t>
         </is>
       </c>
       <c r="D658" t="n">
@@ -13626,12 +13626,12 @@
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>INE040A01034</t>
+          <t>INE758E01017</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="D661" t="n">
@@ -13706,12 +13706,12 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>INE180A01020</t>
+          <t>INE0DYJ01015</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>MFSL</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="D665" t="n">
@@ -13726,12 +13726,12 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>INE0DYJ01015</t>
+          <t>INE180A01020</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>SYRMA</t>
+          <t>MFSL</t>
         </is>
       </c>
       <c r="D666" t="n">
@@ -14546,12 +14546,12 @@
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>INE0NT901020</t>
+          <t>INE158A01026</t>
         </is>
       </c>
       <c r="C707" t="inlineStr">
         <is>
-          <t>NETWEB</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="D707" t="n">
@@ -14566,12 +14566,12 @@
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>INE158A01026</t>
+          <t>INE0NT901020</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>NETWEB</t>
         </is>
       </c>
       <c r="D708" t="n">

</xml_diff>